<commit_message>
Sync architecture to hand-edited fetcher; apply Arial 10pt + col-A-spacer + B2 title conventions; archive stale scaffold_capiq_fetcher
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/broker_fetcher.xlsx
+++ b/templates/broker_fetcher.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Fetcher" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="broker_fetcher_ticker">Fetcher!$B$3</definedName>
+    <definedName name="broker_fetcher_ticker">Fetcher!$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,32 +28,36 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <i val="1"/>
       <color rgb="00808080"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="000000FF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="00000000"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -65,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="000070C0"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,31 +87,24 @@
       <diagonal/>
     </border>
     <border>
-      <left style="dotted">
-        <color rgb="000000FF"/>
-      </left>
-      <right style="dotted">
-        <color rgb="000000FF"/>
-      </right>
-      <top style="dotted">
-        <color rgb="000000FF"/>
-      </top>
-      <bottom style="dotted">
-        <color rgb="000000FF"/>
-      </bottom>
+      <left style="hair"/>
+      <right style="hair"/>
+      <top style="hair"/>
+      <bottom style="hair"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -191,7 +188,7 @@
     <author>scaffold_broker_fetcher</author>
   </authors>
   <commentList>
-    <comment ref="B3" authorId="0" shapeId="0">
+    <comment ref="C6" authorId="0" shapeId="0">
       <text>
         <t>Set this to the ticker you want broker estimates for. CapIQ formulas refresh automatically when you change it (and when fetch_broker_estimates.py drives it programmatically).</t>
       </text>
@@ -489,451 +486,458 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="B2:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="2.71" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="1">
+        <f>broker_fetcher_ticker&amp;" | Broker Estimates Fetcher"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Broker Estimates Fetcher — formulas only. Open in Excel with CapIQ plugin loaded to refresh.</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Run via:</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>python -m shared.fetch_broker_estimates &lt;TICKER&gt;</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Ticker:</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>FY1 fiscal year:</t>
         </is>
       </c>
-      <c r="B4" s="4">
+      <c r="C7" s="5">
         <f>YEAR(IQ_FY1_FYE_DATE(broker_fetcher_ticker))</f>
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>FY2 fiscal year:</t>
         </is>
       </c>
-      <c r="B5" s="4">
+      <c r="C8" s="5">
         <f>YEAR(IQ_FY2_FYE_DATE(broker_fetcher_ticker))</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="9">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>FY3 fiscal year:</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="C9" s="5">
         <f>YEAR(IQ_FY3_FYE_DATE(broker_fetcher_ticker))</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>FY1 Mean</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>FY2 Mean</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>FY3 Mean</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>FY1 High</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>FY1 Low</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>FY1 # Est</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B10" s="4">
+      <c r="C13" s="5">
         <f>IQ_EST_REV(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C10" s="4">
+      <c r="D13" s="5">
         <f>IQ_EST_REV(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D10" s="4">
+      <c r="E13" s="5">
         <f>IQ_EST_REV(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E10" s="4">
+      <c r="F13" s="5">
         <f>IQ_EST_REV_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F10" s="4">
+      <c r="G13" s="5">
         <f>IQ_EST_REV_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G10" s="4">
+      <c r="H13" s="5">
         <f>IQ_EST_NUM_REV(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B11" s="4">
+      <c r="C14" s="5">
         <f>IQ_EST_GP(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C11" s="4">
+      <c r="D14" s="5">
         <f>IQ_EST_GP(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D11" s="4">
+      <c r="E14" s="5">
         <f>IQ_EST_GP(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E11" s="4">
+      <c r="F14" s="5">
         <f>IQ_EST_GP_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="G14" s="5">
         <f>IQ_EST_GP_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G11" s="4">
+      <c r="H14" s="5">
         <f>IQ_EST_NUM_GP(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B12" s="4">
+      <c r="C15" s="5">
         <f>IQ_EST_EBITDA(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C12" s="4">
+      <c r="D15" s="5">
         <f>IQ_EST_EBITDA(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D12" s="4">
+      <c r="E15" s="5">
         <f>IQ_EST_EBITDA(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E12" s="4">
+      <c r="F15" s="5">
         <f>IQ_EST_EBITDA_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F12" s="4">
+      <c r="G15" s="5">
         <f>IQ_EST_EBITDA_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G12" s="4">
+      <c r="H15" s="5">
         <f>IQ_EST_NUM_EBITDA(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B13" s="4">
+      <c r="C16" s="5">
         <f>IQ_EST_EBIT(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C13" s="4">
+      <c r="D16" s="5">
         <f>IQ_EST_EBIT(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D13" s="4">
+      <c r="E16" s="5">
         <f>IQ_EST_EBIT(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E13" s="4">
+      <c r="F16" s="5">
         <f>IQ_EST_EBIT_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F13" s="4">
+      <c r="G16" s="5">
         <f>IQ_EST_EBIT_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G13" s="4">
+      <c r="H16" s="5">
         <f>IQ_EST_NUM_EBIT(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B14" s="4">
+      <c r="C17" s="5">
         <f>IQ_EST_NI(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C14" s="4">
+      <c r="D17" s="5">
         <f>IQ_EST_NI(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D14" s="4">
+      <c r="E17" s="5">
         <f>IQ_EST_NI(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E14" s="4">
+      <c r="F17" s="5">
         <f>IQ_EST_NI_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F14" s="4">
+      <c r="G17" s="5">
         <f>IQ_EST_NI_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G14" s="4">
+      <c r="H17" s="5">
         <f>IQ_EST_NUM_NI(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>EPS (Diluted)</t>
         </is>
       </c>
-      <c r="B15" s="4">
+      <c r="C18" s="5">
         <f>IQ_EST_EPS(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
-      <c r="C15" s="4">
+      <c r="D18" s="5">
         <f>IQ_EST_EPS(broker_fetcher_ticker,IQ_FY2)</f>
         <v/>
       </c>
-      <c r="D15" s="4">
+      <c r="E18" s="5">
         <f>IQ_EST_EPS(broker_fetcher_ticker,IQ_FY3)</f>
         <v/>
       </c>
-      <c r="E15" s="4">
+      <c r="F18" s="5">
         <f>IQ_EST_EPS_HIGH(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
-      <c r="F15" s="4">
+      <c r="G18" s="5">
         <f>IQ_EST_EPS_LOW(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
-      <c r="G15" s="4">
+      <c r="H18" s="5">
         <f>IQ_EST_NUM_EPS(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="B16" s="4">
+      <c r="C19" s="5">
         <f>IQ_EST_CFO(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C16" s="4">
+      <c r="D19" s="5">
         <f>IQ_EST_CFO(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D16" s="4">
+      <c r="E19" s="5">
         <f>IQ_EST_CFO(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E16" s="4">
+      <c r="F19" s="5">
         <f>IQ_EST_CFO_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F16" s="4">
+      <c r="G19" s="5">
         <f>IQ_EST_CFO_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G16" s="4">
+      <c r="H19" s="5">
         <f>IQ_EST_NUM_CFO(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>CapEx</t>
         </is>
       </c>
-      <c r="B17" s="4">
+      <c r="C20" s="5">
         <f>IQ_EST_CAPEX(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="C17" s="4">
+      <c r="D20" s="5">
         <f>IQ_EST_CAPEX(broker_fetcher_ticker,IQ_FY2,IQ_USD)</f>
         <v/>
       </c>
-      <c r="D17" s="4">
+      <c r="E20" s="5">
         <f>IQ_EST_CAPEX(broker_fetcher_ticker,IQ_FY3,IQ_USD)</f>
         <v/>
       </c>
-      <c r="E17" s="4">
+      <c r="F20" s="5">
         <f>IQ_EST_CAPEX_HIGH(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="F17" s="4">
+      <c r="G20" s="5">
         <f>IQ_EST_CAPEX_LOW(broker_fetcher_ticker,IQ_FY1,IQ_USD)</f>
         <v/>
       </c>
-      <c r="G17" s="4">
+      <c r="H20" s="5">
         <f>IQ_EST_NUM_CAPEX(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Revenue Growth FY1 %</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Revenue Growth FY2 %</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Revenue Growth FY3 %</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Gross Margin FY1 %</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>EBITDA Margin FY1 %</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>EBIT Margin FY1 %</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Number of Analysts Covering</t>
         </is>
       </c>
-      <c r="B28" s="4">
+      <c r="C31" s="5">
         <f>IQ_EST_NUM_REV(broker_fetcher_ticker,IQ_FY1)</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Average Price Target</t>
         </is>
       </c>
-      <c r="B29" s="4">
+      <c r="C32" s="5">
         <f>IQ_PRICETARGET_AVG(broker_fetcher_ticker)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Implied Upside %</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Average Recommendation (1=Buy,5=Sell)</t>
         </is>
       </c>
-      <c r="B31" s="4">
+      <c r="C34" s="5">
         <f>IQ_RECOMMENDATION_AVG(broker_fetcher_ticker)</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Recommendation Distribution</t>
         </is>

</xml_diff>